<commit_message>
Add Tier S-A Jobs and realistic 2nd job options sheet
</commit_message>
<xml_diff>
--- a/Work_and_Travel_Master_Job_Database_2027_Clean.xlsx
+++ b/Work_and_Travel_Master_Job_Database_2027_Clean.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WAT 2027 Jobs Masterlist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier S-A Jobs &amp; 2nd Options" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +37,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +54,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAFC"/>
         <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F2FE"/>
+        <bgColor rgb="00E0F2FE"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -93,11 +106,35 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -464,18 +501,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="37" customWidth="1" min="3" max="3"/>
-    <col width="54" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="132" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="132" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,25 +539,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>เวลาทำงานจริง (ช่วงปกติ / ช่วงพีค)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>ค่าแรงฐาน / OT ($/ชม.)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ทิป ($/สัปดาห์)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ชั่วโมงทำงานจริง (คิดเผื่อหัว-ท้ายซีซัน)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ค่าที่พัก ($/สัปดาห์)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>สวัสดิการ (อาหาร ฟรี หรือ อื่นๆ)</t>
         </is>
@@ -546,74 +589,86 @@
           <t>Housekeeping / Room Attendant</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:30 – 15:30 น. (8 ชม.)
+พีค: 07:00 – 17:30 น. (10 ชม. ควงกะ)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>$15 - $30</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>50 – 54 ชม./สัปดาห์ (พีค 58-62 ชม. / หัวท้าย 35-42 ชม.)</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR ตักไม่อั้น 7 วัน, ทิปหัวเตียง, รถรับส่งพนักงาน, ส่วนลดทัวร์/รถไฟ 50%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Denali Princess Wilderness Lodge</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Alaska (AK)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Acadex, OEG, IEE, Higher</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Kitchen Stewarding / Dishwasher (ล้างจาน)</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 16:00 – 00:00 น. (8 ชม.)
+พีค: 15:00 – 01:30 น. (10.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>50 – 55 ชม./สัปดาห์ (ควงกะค่ำได้ง่าย)</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>อาหารบุฟเฟต์ 3 มื้อใน EDR + เชฟทำสเต๊ก/เบอร์เกอร์เลี้ยงในครัวฟรีทุกกะ</t>
         </is>
@@ -640,74 +695,86 @@
           <t>Luggage Handler (พนักงานยกกระเป๋าทัวร์)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 น. หรือ 12:00 – 20:30 น.
+พีค: 07:00 – 18:30 น. (ตามรอบรถไฟ)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>$40 - $70</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>46 – 52 ชม./สัปดาห์</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, ทิปเงินสดจากกรุ๊ปทัวร์ผู้สูงอายุ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Denali Princess Wilderness Lodge</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Alaska (AK)</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>ขอทำเพิ่มหน้างาน (Internal 2nd Job)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Fleet Detailer (งานเสริมล้างรถทัวร์กะดึก 21:00-01:30)</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Fleet Detailer (งานเสริมล้างรถทัวร์กะดึก)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 21:00 – 01:30 น. (4.5 ชม.)
+พีค: 21:00 – 02:30 น. (5.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>คิดเรต OT $24.00/ชม. ทันที</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>20 – 25 ชม./สัปดาห์ (ทำควบหลังงานหลักแม่บ้าน)</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>นับเป็นชั่วโมง OT $24.00 ทั้งหมด, ทำงานในอู่รถบัส Princess, อาหาร EDR 3 มื้อ</t>
         </is>
@@ -734,74 +801,86 @@
           <t>Housekeeping / Laundry</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 น. (8 ชม.)
+พีค: 08:00 – 17:00 น. (9 ชม.)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>40 – 45 ชม./สัปดาห์ (หัวท้าย 32-38 ชม.)</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>$140</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป (ครบสัญญา), รถชัตเติลบัสขึ้น-ลงเขา Sugarloaf, ส่วนลดอาหารร้าน The Perk</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Grande Denali Lodge</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Alaska (AK)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Acadex Thailand</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Housekeeping / Public Area Cleaner</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 น. (8 ชม.)
+พีค: 07:30 – 17:00 น. (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>42 – 46 ชม./สัปดาห์ (หัวท้าย 35-40 ชม.)</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>$140</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป (ครบสัญญา), โรงแรมหรู 4 ดาว, รถชัตเติลบัส, ส่วนลดอาหารห้องอาหาร Alpenglow</t>
         </is>
@@ -828,74 +907,86 @@
           <t>Busser / Food Runner (Alpenglow Restaurant)</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 16:30 – 22:30 น. (6 ชม.)
+พีค: 16:00 – 23:30 น. (7.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>ฐาน $14.00 / OT $21.00</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>$200 - $350</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>40 – 45 ชม./สัปดาห์</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>$140</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>โบนัสพิเศษ +$1.00/ชม. ท้ายทริป, ทิปเงินสดจากแขกไฮเอนด์ร้านอาหารวิวพาโนรามา ($40-$70/คืน)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Mt. McKinley Princess Lodge</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Alaska (AK)</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Higher, OEG, Acadex</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Housekeeping / Kitchen / Laundry</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 น. (8 ชม.)
+พีค: 07:30 – 17:00 น. (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>$10 - $20</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>44 – 48 ชม./สัปดาห์ (หัวท้าย 35-40 ชม.)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, รถรับส่งพนักงาน, ชมวิวยอดเขาเดนาลี บรรยากาศสงบ</t>
         </is>
@@ -922,74 +1013,86 @@
           <t>Food Runner / Laundry / Steward</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 06:30 – 14:30 น. หรือ 15:00 – 23:00 น.
+พีค: กะสลับตามรอบรถไฟ/เครื่องบิน 8 ชม.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>ฐาน $15.50 / OT $23.25</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>$20 - $40</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>36 – 40 ชม./สัปดาห์ (ไม่ค่อยมี OT)</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>หอพักในเมืองแฟร์แบงก์ส + รถชัตเติลบัส, ใกล้ Walmart และร้านอาหารไทย หางาน 2 ง่าย</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Grand Teton Lodge Company (GTLC)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Wyoming (WY)</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Acadex, Higher, OEG, IEE</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Housekeeping / Crew Member</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 น. (8 ชม.)
+พีค: 07:00 – 17:30 น. (10 ชม. ควงกะ)</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>ฐาน $17.75 / OT $26.62</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>54 – 60 ชม./สัปดาห์ (พีค 60-64 ชม. / หัวท้าย 40 ชม.)</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>หอพักฟรี 100%! + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), ส่วนลดซื้อของ 40%, เข้าอุทยาน Grand Teton &amp; Yellowstone ฟรี</t>
         </is>
@@ -1016,74 +1119,86 @@
           <t>Kitchen Crew / Dishwasher / Food Prep</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 06:00 – 14:30 น. หรือ 15:00 – 23:00 น.
+พีค: 14:00 – 00:30 น. (ช่วยจัดเลี้ยง Banquet)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>ฐาน $17.75 / OT $26.62</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>52 – 58 ชม./สัปดาห์ (ควงกะ Banquet ได้)</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>$0</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>หอพักฟรี 100%! + อาหาร 3 มื้อ EDR + กินฟรีในครัว, สิทธิประโยชน์เครือ Vail Resorts</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Xanterra Yellowstone Lodges</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Wyoming/MT</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>OEG, IEE Thailand</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Hospitality Crew / Kitchen / Steward</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:00 – 15:30 น. หรือ 15:00 – 23:30 น.
+พีค: 06:30 – 16:30 น. (10 ชม.)</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>ฐาน $15.70 / OT $23.55</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>46 – 52 ชม./สัปดาห์ (หัวท้าย 38-42 ชม.)</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>$120</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>รวมหอพัก + อาหารบุฟเฟต์ 3 มื้อ EDR, หอพักใหม่ Arnica, เที่ยวบ่อน้ำพุร้อนและไกเซอร์ Yellowstone ฟรี</t>
         </is>
@@ -1110,74 +1225,86 @@
           <t>Housekeeping / Guest Service</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:30 – 16:30 น. (8 ชม.)
+พีค: 08:00 – 17:30 น. (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>ฐาน $16.50 / OT $24.75</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>$50 - $100</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>42 – 46 ชม./สัปดาห์</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>$100</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>แคมป์กระโจมซาฟารีหรู, อาหารพนักงาน, ทิปเงินสดจากแขกไฮเอนด์ บรรยากาศเป็นกันเอง</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Kalahari Resorts &amp; Conventions</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Wisconsin (WI)</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>OEG, Acadex, Higher</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Lifeguard / Housekeeping (งานหลัก)</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 น. หรือ 12:00 – 20:30 น.
+พีค: 09:00 – 19:30 น. (10 ชม.)</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>38 – 44 ชม./สัปดาห์ (เกลี่ยกะ 40 ชม.)</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>$105</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>หอพัก Kalahari Village, บัตรเล่นสวนน้ำฟรี, เมืองปั่นจักรยาน 100%, หางาน 2 ร้านอาหารง่าย</t>
         </is>
@@ -1204,74 +1331,86 @@
           <t>Barback / Busser / Runner (งานที่สอง)</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 17:30 – 22:30 น. (5 ชม.)
+พีค: 17:00 – 00:30 น. (7.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>ฐาน $12.00 – $14.00</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>$250 - $500</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>20 – 25 ชม./สัปดาห์ (กะค่ำ 17:30-23:00)</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>รับทิปเงินสดทุกคืน ยัดกระเป๋ากลับห้องทันที ($50-$100/คืน), อาหารพนักงานในกะ (ทำควบกับงานหลัก)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Dollywood Theme Park &amp; Resorts</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Tennessee (TN)</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>New Step, Acadex</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Ride Operator / Food Service / Retail</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 น. (8 ชม.)
+พีค: 09:00 – 21:30 น. (12 ชม. สวนสนุกเปิดดึก)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>ฐาน $15.00 / OT $22.50</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>44 – 50 ชม./สัปดาห์ (หัวท้าย 35-40 ชม.)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>$110</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>ปลอดภาษีเงินได้รัฐ 0%, นั่งรถราง Pigeon Forge Trolley $1-$2.50/วัน, บัตรเข้าสวนสนุก Dollywood &amp; Splash Country ฟรี</t>
         </is>
@@ -1298,76 +1437,2088 @@
           <t>Pool Lifeguard</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>ปกติ: 10:30 – 19:30 น. (9 ชม.)
+พีค: 10:00 – 20:30 น. (10.5 ชม. สระเปิดยาว)</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>ฐาน $16.00 / OT $24.00</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>50 – 54 ชม./สัปดาห์ (การันตี OT 10-14 ชม.)</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>$120</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>การันตีชั่วโมง OT สม่ำเสมอ 10-14 ชม./สัปดาห์ ไม่ผันผวนตามนักท่องเที่ยว, อพาร์ตเมนต์แชร์กับเพื่อน</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Cedar Point Amusement Park</t>
         </is>
       </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Ohio (OH)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>OEG, IEE Thailand</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Ride Operator / Food Service</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 10:00 – 18:30 น. (8 ชม.)
+พีค: 09:30 – 22:30 น. (12 ชม. สวนสนุกปิดดึก)</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $14.50 / OT $21.75</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>46 – 52 ชม./สัปดาห์ (หัวท้าย 38-42 ชม.)</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>$80</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>หอพักราคาถูกมาก ($80/wk), รถบัสรับส่งฟรี, บัตรเล่นเครื่องเล่นสวนสนุกระดับโลกฟรี</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="41" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tier &amp; รัฐ (State)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ชื่องาน / สถานที่ทำงานหลัก (Employer)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Agency ที่ถือสัญญา</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ตำแหน่งงานหลัก (Role)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>⏱️ เวลาทำงานหลัก (ปกติ / พีค)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ค่าแรงฐาน / OT ($/ชม.)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ทิป ($/สัปดาห์)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ชั่วโมงงานหลัก (ชม./wk)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ค่าที่พัก ($/สัปดาห์)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>สวัสดิการ (อาหาร ฟรี หรือ อื่นๆ)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>🔥 งานที่สองที่ทำต่อได้จริง (ตัวเลือกที่ 1)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>🔥 งานที่สองที่ทำต่อได้จริง (ตัวเลือกที่ 2)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>🔥 งานที่สองที่ทำต่อได้จริง (ตัวเลือกที่ 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Tier S - Alaska (AK)</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Denali Princess Wilderness Lodge</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Acadex, OEG, IEE, Higher</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Housekeeping / Room Attendant</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:30 – 15:30 (8 ชม.)
+พีค: 07:00 – 17:30 (10 ชม. ควงกะ)</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>$15 - $30</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>50 – 54 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR ตักไม่อั้น 7 วัน, ทิปหัวเตียง, รถรับส่งพนักงาน, ส่วนลดทัวร์ 50%</t>
+        </is>
+      </c>
+      <c r="K2" s="10" t="inlineStr">
+        <is>
+          <t>🚌 Fleet Detailer (ในโรงแรม): ล้างรถทัวร์กะดึก 21:00-01:30 น. ได้เรต OT $24.00/ชม. ทันที (ไม่ต้องขอสปอนเซอร์)</t>
+        </is>
+      </c>
+      <c r="L2" s="10" t="inlineStr">
+        <is>
+          <t>🍕 Prospectors Pizzeria: เดิน 10 นาที ล้างจาน/Barback กะค่ำ 18:30-00:30 น. ($15/ชม. + ทิปสด $40-$70/คืน)</t>
+        </is>
+      </c>
+      <c r="M2" s="10" t="inlineStr">
+        <is>
+          <t>🍽️ Fannie Q’s Saloon (ในโรงแรม): ช่วยจัดเลี้ยง/Runner 17:00-22:00 น. ได้เรต OT $24/ชม. + ทิป</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Tier S - Alaska (AK)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Denali Princess Wilderness Lodge</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Acadex, OEG, IEE, Higher</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Kitchen Stewarding / Dishwasher</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 16:00 – 00:00 (8 ชม.)
+พีค: 15:00 – 01:30 (10.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>50 – 55 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>อาหารบุฟเฟต์ 3 มื้อใน EDR + เชฟทำสเต๊ก/เบอร์เกอร์เลี้ยงในครัวฟรีทุกกะ</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>🧹 เช้าช่วยแม่บ้าน (Housekeeping): 08:30-14:30 น. ขอกะเช้าเพิ่มในโรงแรม ได้เรต OT $24/ชม.</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>🧳 Luggage Handler: ช่วยยกกระเป๋ารอบรถไฟเช้า 08:00-12:00 น. ได้ทิปสดจากทัวร์</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>🛍️ Denali Boardwalk Gift Shops: แคชเชียร์/จัดของกะสาย 09:00-14:00 น. ($15/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Tier S - Alaska (AK)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Grande Denali Lodge &amp; Denali Bluffs</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Acadex Thailand</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Housekeeping / Public Area</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 (8 ชม.)
+พีค: 07:30 – 17:00 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>42 – 46 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>$140</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>โบนัส +$1.00/ชม. ท้ายทริป, โรงแรมหรู 4 ดาวบนยอดเขา, รถชัตเติลบัส, ส่วนลดอาหาร</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>🍷 Alpenglow Restaurant (ในโรงแรม): Busser/Food Runner 17:00-23:00 น. ($14/ชม. + ทิปสดเศรษฐี $50-$80/คืน)</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>🥪 Subway Denali / The Black Bear: นั่งชัตเติลลงเขาไปทำกะเย็น 17:00-22:00 น. ($15/ชม.)</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>🍽️ Denali Princess Kitchens: เดินลงเขา 15 นาที ขอล้างจานกะค่ำ 18:00-00:00 น. ($16/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Tier S - Alaska (AK)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Mt. McKinley Princess Lodge</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Higher, OEG, Acadex</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Housekeeping / Kitchen</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 (8 ชม.)
+พีค: 07:30 – 17:00 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>$10 - $20</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>44 – 48 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>อาหารบุฟเฟต์ 3 มื้อฟรีใน EDR, รถรับส่ง, ชมวิวยอดเขาเดนาลี บรรยากาศสงบ</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>🥩 20,320 Alaskan Grill (ในโรงแรม): Busser/Steward กะค่ำ 17:30-22:30 น. (เรต OT $24/ชม. + ทิป)</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>🍕 Northland Wood Fired Pizza (ในโรงแรม): ผู้ช่วยทำพิซซ่า/ครัว 16:30-21:30 น. (เรต OT $24/ชม.)</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>🥐 Talkeetna Roadhouse: นั่งรถตู้พนักงานเข้าเมือง Talkeetna ช่วยล้างจาน/ทำขนมวันหยุด</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Tier S - Alaska (AK)</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Fairbanks Princess Riverside Lodge</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>IEE, Acadex, Higher</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Food Runner / Laundry / Steward</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 06:30 – 14:30 หรือ 15:00 – 23:00
+พีค: กะสลับตามรอบรถไฟ 8 ชม.</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>$20 - $40</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>36 – 40 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>หอพักในเมืองแฟร์แบงก์ส + รถชัตเติลบัส, ใกล้ Walmart และร้านอาหารไทย หางาน 2 ง่าย</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>🛒 Walmart Supercenter Fairbanks: จัดสต็อกสินค้า/แคชเชียร์ 16:30-22:30 น. ($16-$17/ชม. มีรถเมล์ผ่าน)</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>🍜 Pad Thai Restaurant / Thai House: ผู้ช่วยครัว/เสิร์ฟ 17:00-22:30 น. (มีทิปสด + กินอาหารไทยฟรี)</t>
+        </is>
+      </c>
+      <c r="M6" s="10" t="inlineStr">
+        <is>
+          <t>🍺 The Pump House Restaurant: Busser/Dishwasher ร้านอาหารริมแม่น้ำชื่อดัง 17:30-23:00 น. ($15/ชม. + ทิป)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Tier S - Wyoming (WY)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Grand Teton Lodge Company (GTLC)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Acadex, Higher, OEG, IEE</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Housekeeping / Crew Member</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 (8 ชม.)
+พีค: 07:00 – 17:30 (10 ชม. ควงกะ)</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $17.75 / OT $26.62</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>54 – 60 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>$0 (ฟรี!)</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>หอพักฟรี 100%! + อาหารบุฟเฟต์ 3 มื้อ EDR ($105/wk), ส่วนลด 40%, บัตรผ่าน 2 อุทยานฟรี</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>🍽️ Mural Room &amp; Pioneer Grill (ในโรงแรม): Busser/Steward 17:30-22:30 น. ได้เรต OT $26.62/ชม. + ทิป</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>🍸 Blue Heron Lounge (ในโรงแรม): Barback ช่วยยกน้ำแข็ง/ล้างแก้ว 18:00-23:30 น. (เรต OT $26.62 + Tip-Out)</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>🛶 Colter Bay Chuckwagon &amp; Marina: นั่งชัตเติลฟรีไปช่วยร้านอาหาร/มินิมาร์ทริมทะเลสาบ 17:00-21:30 น.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Tier S - Wyoming (WY)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Xanterra Yellowstone Lodges</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>OEG, IEE Thailand</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Hospitality Crew / Kitchen Steward</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:00 – 15:30 หรือ 15:00 – 23:30
+พีค: 06:30 – 16:30 (10 ชม.)</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $15.70 / OT $23.55</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>46 – 52 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>$120 (รวมกิน)</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>รวมหอพัก + อาหารบุฟเฟต์ 3 มื้อ EDR, หอพักใหม่ Arnica, เที่ยวบ่อน้ำพุร้อน Yellowstone ฟรี</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>🌋 Old Faithful Snow Lodge Dining: Busser/Steward กะค่ำ 17:00-22:30 น. (เรต OT $23.55/ชม. + ทิป)</t>
+        </is>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>🛍️ Delaware North General Stores: แคชเชียร์ร้านของฝากข้างๆ เดิน 3 นาที 17:00-21:30 น. ($15.50/ชม.)</t>
+        </is>
+      </c>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>🍻 Employee Pub &amp; Rec Hall: ผู้ช่วยดูแลผับพนักงาน/ทำความสะอาดรอบดึก 19:30-23:30 น.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Tier S - Wyoming (WY)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Under Canvas Grand Teton / Yellowstone</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Higher Education</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Housekeeping / Guest Service</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:30 – 16:30 (8 ชม.)
+พีค: 08:00 – 17:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $16.50 / OT $24.75</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>$50 - $100</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>42 – 46 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>แคมป์กระโจมซาฟารีหรู, อาหารพนักงาน, ทิปเงินสดจากแขกไฮเอนด์ บรรยากาศเป็นกันเอง</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>🏕️ Embers Restaurant (ในแกลมปิ้ง): Food Runner กะค่ำ 17:30-22:00 น. (ได้ทิปสดคืนละ $40-$60)</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>☕ Moose-Wilson Road Cafes: ผู้ช่วยบาริสต้า/เบเกอรี่ช่วงเช้าตรู่ 06:00-08:00 น. หรือเย็น</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>🛒 Jackson Town Local Diners: นั่งรถเข้าเมืองแจ็กสัน ทำงานร้านอาหารวันหยุด</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Tier S - Wyoming (WY)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Four Seasons Resort / Snake River Lodge</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>OEG, Acadex</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Housekeeping / Stewarding</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 (8 ชม.)
+พีค: 07:30 – 17:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $17.50 / OT $26.25</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>45 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>$140</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>รีสอร์ตหรู 5 ดาวใน Teton Village, หอพักพนักงาน, นั่งรถบัส START Bus ฟรี</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>🍺 The Mangy Moose Saloon (Teton Village): Barback/Busser ร้านผับดัง 18:00-00:30 น. (ทิปสด $60-$120/คืน)</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>🤠 Million Dollar Cowboy Bar (เมือง Jackson): นั่ง START Bus เข้าเมือง ทำ Barback 19:00-01:30 น.</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>🍕 Alpenhof Bistro: ล้างจาน/ผู้ช่วยครัว 17:30-22:30 น. ($16/ชม. + อาหารฟรี)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Tier S - Wisconsin (WI)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Kalahari Resorts &amp; Conventions</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>OEG, Acadex, Higher</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Lifeguard / Housekeeping</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 หรือ 12:00 – 20:30
+พีค: 09:00 – 19:30 (10 ชม.)</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>38 – 44 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>หอพัก Kalahari Village, บัตรเล่นสวนน้ำฟรี, เมืองปั่นจักรยาน 100%, หางาน 2 ง่ายที่สุดในอเมริกา</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>🍕 Moosejaw Pizza &amp; Dells Brewing: ปั่นจักรยาน 10 นาที Busser/Barback 18:30-23:30 น. ($13/ชม. + ทิปสด $60-$90/คืน)</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>🍔 Buffalo Phil’s Grille: Food Runner/Busser เสิร์ฟอาหารด้วยรถไฟจิ๋ว 18:00-22:30 น. ($13/ชม. + ทิปสด $50-$80)</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>🧀 MACS Macaroni &amp; Cheese / Dairy Queen: แคชเชียร์/ครัวกะดึก 18:30-23:00 น. ($14.50-$15.50/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Tier S - Wisconsin (WI)</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Noah’s Ark Waterpark</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>OEG, IEE, New Step</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Ride Operator / Park Services</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:00 – 17:30 (8 ชม.)
+พีค: 08:30 – 18:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $14.50 / OT $21.75</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>40 – 46 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>สวนน้ำกลางแจ้งใหญ่ที่สุดในอเมริกา, เล่นสวนน้ำฟรี, หอพักพนักงานใกล้ที่ทำงาน</t>
+        </is>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>🍻 Monk’s Bar &amp; Grill (Downtown Dells): ปั่นจักรยานไปทำ Barback/Busser 18:30-00:00 น. (ทิปสดแน่นมาก)</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>🌭 Hot Dog Avenue / Brat House: แคชเชียร์/ครัวปิด 18:00-22:30 น. ($14.50/ชม. + กินฟรี)</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>🥞 Paul Bunyan’s Cook Shanty: ช่วยล้างจาน/ทำความสะอาดรอบค่ำ 17:30-22:00 น.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Tier S - Wisconsin (WI)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Chula Vista Resort &amp; Waterpark</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Higher, Acadex, IEE</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Housekeeping / Lifeguard</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:30 – 16:30 (8 ชม.)
+พีค: 08:00 – 17:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>40 – 45 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>รีสอร์ตริมแม่น้ำ Wisconsin River, สวนน้ำในร่ม/กลางแจ้ง, หอพักในรีสอร์ต</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>🥩 Kaminski’s Chop House (ในรีสอร์ต): Busser ร้านสเต๊กหรู 17:30-23:00 น. ($12/ชม. + ทิปสดเศรษฐี $70-$120/คืน)</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>🌮 Mexicali Rose: Busser/Runner ร้านอาหารเม็กซิกันริมน้ำ 18:00-23:00 น. ($13/ชม. + ทิปสด)</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>🍕 Kilbourn City Grill (ในรีสอร์ต): ล้างจาน/ผู้ช่วยครัว 17:00-22:00 น. (ขอ OT ในรีสอร์ตได้)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Tier S - Tennessee (TN)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Dollywood Theme Park &amp; Splash Country</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>New Step, Acadex</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Ride Operator / Food Service / Retail</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 (8 ชม.)
+พีค: 09:00 – 21:30 (12 ชม. สวนสนุกเปิดดึก)</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>44 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>$110</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>ปลอดภาษีเงินได้รัฐ 0%, นั่งรถราง Pigeon Forge Trolley $1/วัน, บัตรเข้าสวนสนุก Dollywood ฟรี</t>
+        </is>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>🍗 Paula Deen’s Family Kitchen (The Island): นั่งรถรางไปทำ Busser/Steward 18:30-23:00 น. ($13/ชม. + ทิปสด $60-$90)</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>🍕 Mellow Mushroom Pizza: Barback/Busser ร้านพิซซ่าคราฟต์เบียร์ 18:30-00:00 น. ($12/ชม. + ทิปสด $50-$80)</t>
+        </is>
+      </c>
+      <c r="M14" s="10" t="inlineStr">
+        <is>
+          <t>🥞 Puckett’s Grocery &amp; Restaurant: Food Runner/Busser 18:00-23:00 น. ($13/ชม. + ทิป)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Tier S - Tennessee (TN)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Wilderness at the Smokies</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>OEG, Acadex, Higher</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Lifeguard / Housekeeping</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:00 – 17:30 (8 ชม.)
+พีค: 08:30 – 19:30 (10.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>42 – 48 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>สวนน้ำในร่มใหญ่ที่สุดในเทนเนสซี, ปลอดภาษีรัฐ 0%, หอพักพนักงาน Sevierville</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>🍏 Applewood Farmhouse Restaurant: Busser/Runner ร้านอาหารชื่อดังคนแน่นมาก 18:00-22:30 น. (ทิปสด $60-$100/คืน)</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>🥩 Hidden Trail Restaurant (ในรีสอร์ต): ล้างจาน/Busser กะค่ำ 18:00-22:30 น. (ขอ OT ในรีสอร์ต $22.50/ชม.)</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>🛍️ Tanger Outlets Sevierville: พนักงานจัดสต็อกสินค้า/ปิดร้าน 18:00-21:30 น. ($15/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Tier S - Tennessee (TN)</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Ober Mountain / Gatlinburg SkyPark Area</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>IEE, New Step</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Attractions Operator / Retail</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:00 – 17:00 (8 ชม.)
+พีค: 08:30 – 19:00 (10 ชม.)</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>40 – 46 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>$110</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>กระเช้าลอยฟ้าและสวนสนุกบนยอดเขา Gatlinburg, ปลอดภาษีรัฐ 0%, เมืองเดินเท้า 100%</t>
+        </is>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
+        <is>
+          <t>🍻 Smoky Mountain Brewery (Gatlinburg): เดินลงเขามาทำ Barback 18:00-00:30 น. ($12/ชม. + ทิปสด $70-$120/คืน)</t>
+        </is>
+      </c>
+      <c r="L16" s="10" t="inlineStr">
+        <is>
+          <t>🥩 Alamo Steakhouse: Busser/Dishwasher ร้านสเต๊กคาวบอย 17:30-23:00 น. ($13/ชม. + ทิป)</t>
+        </is>
+      </c>
+      <c r="M16" s="10" t="inlineStr">
+        <is>
+          <t>🥃 Ole Smoky Moonshine Distillery: พนักงานเช็ดแก้ว/เติมสต็อก/แคชเชียร์ 17:30-22:30 น. ($15/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Tier S - Texas (TX)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Schlitterbahn Waterpark (New Braunfels)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>OEG, Acadex, IEE</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Lifeguard / Park Operations</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 (8 ชม.)
+พีค: 09:00 – 19:30 (10 ชม.)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>44 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>$110</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>สวนน้ำระดับตำนานของเท็กซัส, ปลอดภาษีเงินได้รัฐ 0%, เล่นสวนน้ำฟรี</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>🥩 Gristmill River Restaurant (Gruene): Busser ร้านอาหารริมแม่น้ำสุดคึกคัก 18:30-23:30 น. ($12/ชม. + ทิปสด $60-$100)</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>🦫 Buc-ee’s New Braunfels (ใหญ่ที่สุดในโลก): แคชเชียร์/Food Prep กะดึก 19:00-00:00 น. ($17-$19/ชม. จ่ายหนักมาก)</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>🍺 Krause’s Cafe &amp; Biergarten: Barback/Runner ร้านเบียร์เยอรมัน 18:00-23:00 น. ($13/ชม. + ทิป)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Tier A - Montana (MT)</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Glacier National Park Lodges (Pursuit/Xanterra)</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>OEG, Acadex, Higher</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Hospitality Crew / Housekeeping</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 (8 ชม.)
+พีค: 07:30 – 17:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>46 – 52 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>$115 (รวมกิน)</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>อุทยานธรรมชาติธารน้ำแข็ง Glacier NP, ปลอดภาษีมูลค่าเพิ่ม 0% Sales Tax, หอพัก+อาหาร EDR</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>🥩 Belton Chalet Dining Room: Busser/Steward ร้านอาหารประวัติศาสตร์ 17:30-22:30 น. ($15/ชม. + ทิป)</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>🛶 Glacier Raft Company Base: พนักงานล้างทำความสะอาดเรือยาง/อุปกรณ์ล่องแกแก่ง 17:00-21:30 น. ($16/ชม.)</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr">
+        <is>
+          <t>🥐 West Glacier Bakery &amp; Cafe: ผู้ช่วยเตรียมวัตถุดิบ/ล้างจาน 17:00-22:00 น.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Tier A - Montana (MT)</t>
+        </is>
+      </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Ohio (OH)</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
+          <t>Big Sky Resort / Montage Big Sky</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Acadex, Higher, IEE</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Mountain Operations / Housekeeping</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:30 (8 ชม.)
+พีค: 07:30 – 17:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $17.50 / OT $26.25</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>46 – 52 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>$140</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>รีสอร์ตภูเขาหรูหราไฮเอนด์, ค่าแรงฐานสูงมาก, มีรถบัส Skyline Bus ฟรี</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>🍺 Lone Peak Brewery (Town Center): Barback/Busser 17:30-23:30 น. ($15/ชม. + ทิปสดเศรษฐี $60-$100/คืน)</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>🍖 The Riverhouse BBQ: Busser/Runner ร้านบาร์บีคิวริมแม่น้ำ Gallatin 17:00-22:30 น. ($14/ชม. + ทิป)</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>🛒 Roxy’s Market Big Sky: พนักงานจัดสต็อกซูเปอร์มาร์เก็ต 18:00-22:00 น. ($17/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Tier A - Maryland (MD)</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Premier Aquatics / High Sierra Pools</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Acadex, New Step, ALC</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Pool Lifeguard (Bethesda/Rockville)</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>ปกติ: 10:30 – 19:30 (9 ชม.)
+พีค: 10:00 – 20:30 (10.5 ชม. สระเปิดยาว)</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>50 – 54 ชม./wk (การันตี OT)</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>$120</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>การันตีชั่วโมง OT แน่นอนสัปดาห์ละ 10-14 ชม., อพาร์ตเมนต์แชร์กับเพื่อน, รถไฟใต้ดิน Metro เข้า DC</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>🛒 Giant Food / Safeway: พนักงานจัดสต็อกสินค้ากะดึก 20:30-01:00 น. ($16-$17.50/ชม. มีสาขาใกล้ที่พัก)</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>🍜 Thai Tanic / Ruan Thai (Bethesda/Silver Spring): ผู้ช่วยครัว/แพ็กอาหาร 20:00-23:30 น. (มีอาหารไทยฟรี)</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="inlineStr">
+        <is>
+          <t>🎯 Target / CVS Pharmacy: แคชเชียร์/ปิดร้าน 20:00-23:30 น. ($16.00/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Tier A - Maryland (MD)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Ocean City Boardwalk Hotels &amp; Resorts</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>IEE, New Step, OEG</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Housekeeping / Ride Operator</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:30 – 16:30 (8 ชม.)
+พีค: 08:00 – 17:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>44 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>$125</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>เมืองตากอากาศชายหาด Atlantic, รถบัส Coastal Highway วิ่ง 24 ชม., หางานสองง่ายมาก</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>🌴 Seacrets Jamaica USA (ผับริมหาดยักษ์ใหญ่): Barback/Busser 18:00-01:30 น. ($12/ชม. + ทิปสดมหาศาล $80-$150/คืน)</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>🍟 Thrasher’s French Fries (ริม Boardwalk): แคชเชียร์/ทอดเฟรนช์ฟรายส์ 18:00-23:00 น. ($15/ชม.)</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>🍺 Shenanigans Irish Pub: ล้างจาน/ผู้ช่วยบาร์ 18:30-00:30 น. ($14/ชม. + ทิป)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Tier A - South Dakota (SD)</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Xanterra Mount Rushmore / Keystone Lodges</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>OEG, IEE, Higher</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Retail / Food Service / Housekeeping</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:30 – 16:30 (8 ชม.)
+พีค: 08:00 – 17:30 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>44 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>$105</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>ทำงานหน้าอนุสรณ์สถานแห่งชาติ Mount Rushmore, ปลอดภาษีรัฐ 0%, หอพัก+อาหาร EDR</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>🍔 Carver’s Cafe at Mt Rushmore: ล้างจาน/ปิดครัว 17:00-21:30 น. (ขอ OT ในอุทยาน $23.25/ชม.)</t>
+        </is>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>🥩 Ruby House Restaurant (Keystone): Busser ร้านอาหารธีมคาวบอยย้อนยุค 17:30-22:30 น. ($13/ชม. + ทิป)</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="inlineStr">
+        <is>
+          <t>🚂 1880 Train / Keystone Gift Shops: พนักงานร้านของฝาก/สถานีรถไฟโบราณ 17:00-21:30 น. ($15/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Tier A - South Dakota (SD)</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Custer State Park Resorts (State Game Lodge)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Higher, Acadex</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Guest Service / Housekeeping</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:30 – 15:30 (8 ชม.)
+พีค: 07:00 – 16:30 (9 ชม.)</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>42 – 48 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>$105 (รวมกิน)</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>อุทยานธรรมชาติฝูงควายไบซัน Custer SP, ปลอดภาษีรัฐ 0%, หอพัก+อาหาร EDR</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>🥩 State Game Lodge Dining Room: Busser ร้านสเต๊กควายไบซันหรู 17:00-22:00 น. ($13/ชม. + ทิปสด $50-$80)</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>🍔 Black Hills Burger &amp; Bun (เมือง Custer): ล้างจาน/ครัว 17:00-21:30 น. ($15/ชม. + กินฟรี)</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>🏕️ Sylvan Lake General Store: พนักงานมินิมาร์ท/เช่าเรือแคนู 16:30-21:00 น.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Tier A - Utah (UT)</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Zion National Park Lodge (Xanterra Springdale)</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>OEG, IEE, Acadex</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Hospitality Crew / Housekeeping</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:30 – 15:30 (8 ชม.)
+พีค: 07:00 – 16:30 (9 ชม.)</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>ฐาน $16.00 / OT $24.00</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>44 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>$110</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>อุทยานแห่งชาติหุบเขาผาแดง Zion NP, มีรถชัตเติลบัสฟรีวิ่งตลอดถนน Springdale</t>
+        </is>
+      </c>
+      <c r="K24" s="13" t="inlineStr">
+        <is>
+          <t>🌮 Bit &amp; Spur Restaurant &amp; Saloon: Busser/Barback 17:30-23:00 น. ($13/ชม. + ทิปสดแขกต่างชาติ $50-$90/คืน)</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>🍔 Oscar’s Cafe (Springdale): Food Runner/Busser 17:00-22:00 น. ($13/ชม. + ทิป)</t>
+        </is>
+      </c>
+      <c r="M24" s="13" t="inlineStr">
+        <is>
+          <t>🍺 Zion Canyon Brew Pub: ล้างจาน/ผู้ช่วยครัวหน้าปากทางเข้าอุทยาน 18:00-23:30 น. ($15/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Tier A - Utah (UT)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Ruby’s Inn / Bryce Canyon Grand Hotel</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Higher, IEE, Acadex</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Housekeeping / Fast Food / Retail</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 (8 ชม.)
+พีค: 07:30 – 17:00 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $15.00 / OT $22.50</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>42 – 48 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>อาณาจักรโรงแรมและรีสอร์ต Ruby’s Inn หน้าปากทาง Bryce Canyon NP, หอพักพนักงานใกล้ที่ทำงาน</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>🥩 Cowboy’s Buffet &amp; Steak Room (ในเครือ): Busser/Steward 17:00-22:30 น. (ขอ OT ในเครือ $22.50/ชม.)</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>🤠 Ebenezer’s Barn &amp; Grill: Food Runner งานดินเนอร์โชว์คาวบอย 18:00-22:00 น. (ได้ส่วนแบ่งทิป)</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>🛒 Ruby’s General Store &amp; Diner: แคชเชียร์/ผู้ช่วยครัว 17:00-21:30 น. ($15/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Tier A - Maine (ME)</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Bar Harbor Grand Hotel / Harborside Hotel</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Acadex, OEG, Higher</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Housekeeping / Laundry</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>ปกติ: 08:00 – 16:00 (8 ชม.)
+พีค: 07:30 – 17:00 (9.5 ชม.)</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>ฐาน $16.50 / OT $24.75</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>44 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>$130</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
+        <is>
+          <t>เมืองตากอากาศชายทะเล Bar Harbor &amp; อุทยาน Acadia NP, รถบัส Island Explorer ฟรี</t>
+        </is>
+      </c>
+      <c r="K26" s="13" t="inlineStr">
+        <is>
+          <t>🦞 Stewman’s Lobster Pound (ริมทะเล): Busser/Barback ร้านกุ้งล็อบสเตอร์ 17:30-23:00 น. ($13/ชม. + ทิปสด $60-$120/คืน)</t>
+        </is>
+      </c>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t>🍺 Geddy’s Down Under / The Chart Room: Busser/Runner 18:00-23:30 น. (ทิปสดแน่นมาก)</t>
+        </is>
+      </c>
+      <c r="M26" s="13" t="inlineStr">
+        <is>
+          <t>🍦 Ben &amp; Bill’s Chocolate Emporium: พนักงานตักไอศกรีม/แคชเชียร์ 17:00-22:00 น. ($15.50/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Tier A - Ohio (OH)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Cedar Point Amusement Park &amp; Resorts</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>OEG, IEE Thailand</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Ride Operator / Food Service</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 10:00 – 18:30 (8 ชม.)
+พีค: 09:30 – 22:30 (12 ชม. สวนสนุกปิดดึก)</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>ฐาน $14.50 / OT $21.75</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>46 – 52 ชม./สัปดาห์ (หัวท้าย 38-42 ชม.)</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>$80</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>หอพักราคาถูกมาก ($80/wk), รถบัสรับส่งฟรี, บัตรเล่นเครื่องเล่นสวนสนุกระดับโลกฟรี</t>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>46 – 52 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>$80 (ถูกสุด)</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>สวนสนุกเครื่องเล่นระดับโลก, หอพักราคาถูกที่สุดในอเมริกา ($80/wk), รถบัสรับส่งฟรี, เล่นสวนสนุกฟรี</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>🏨 Hotel Breakers / Castaway Bay (ในสวนสนุก): ล้างจาน/แม่บ้านกะค่ำ 19:00-00:00 น. (ขอ OT ในสวนสนุก $21.75/ชม.)</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>🍖 Famous Dave’s BBQ (Cedar Point Marina): Busser/Dishwasher 18:30-23:30 น. ($13/ชม. + ทิปสด)</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
+          <t>🐴 Thirsty Pony / Kalahari Sandusky: Barback/Busser ร้านอาหารใกล้เคียง 19:00-00:30 น.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Tier A - Colorado (CO)</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>YMCA of the Rockies (Estes Park Center)</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Higher, IEE, Acadex</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Housekeeping / Food Service</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>ปกติ: 07:30 – 15:30 (8 ชม.)
+พีค: 07:00 – 16:30 (9 ชม.)</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>ฐาน $15.50 / OT $23.25</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>42 – 48 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>$110 (รวมกิน)</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>แคมป์รีสอร์ตกลางเทือกเขา Rocky Mountain NP, หอพัก+อาหารบุฟเฟต์ 3 มื้อ, รถชัตเติลบัสเข้าเมืองฟรี</t>
+        </is>
+      </c>
+      <c r="K28" s="13" t="inlineStr">
+        <is>
+          <t>🏨 The Stanley Hotel (โรงแรมประวัติศาสตร์ The Shining): Busser/Steward ร้านอาหารหรู 17:30-23:00 น. (ทิปสด $50-$90)</t>
+        </is>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>🍔 Penelope’s Old Time Burgers: ผู้ช่วยครัว/ทอดเบอร์เกอร์ 17:00-21:30 น. ($15/ชม. + กินฟรี)</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="inlineStr">
+        <is>
+          <t>🍺 Estes Park Brewery / Rock Cut Brewing: ล้างแก้ว/ผู้ช่วยบาร์ 18:00-22:30 น. ($15/ชม.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Tier A - Virginia (VA)</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Busch Gardens Williamsburg / Water Country</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>New Step, Acadex</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Ride Operator / Culinary Operations</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>ปกติ: 09:30 – 18:00 (8 ชม.)
+พีค: 09:00 – 21:30 (12 ชม. สวนสนุกเปิดดึก)</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>ฐาน $14.50 / OT $21.75</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>44 – 50 ชม./wk</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>$115</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>สวนสนุกธีมยุโรปชื่อดัง, บัตรเข้าสวนสนุกและสวนน้ำฟรี, หอพักพนักงาน Williamsburg</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>🏰 Kingsmill Resort (ริมแม่น้ำ James River): Banquet Server/Busser งานจัดเลี้ยง 18:30-23:00 น. (ทิปสด $50-$90/คืน)</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>🦀 Captain George’s Seafood Buffet: Busser/Dishwasher บุฟเฟต์ซีฟู้ดยักษ์ใหญ่ 18:30-23:30 น. (คนแน่นมาก ทิปดี)</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>🥞 Cracker Barrel / Pancake House: ผู้ช่วยครัว/ล้างจานรอบค่ำ 18:00-22:00 น. ($14.50/ชม.)</t>
         </is>
       </c>
     </row>

</xml_diff>